<commit_message>
Admin: edit data/events.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -507,7 +507,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>previous</v>
+        <v/>
       </c>
       <c r="B3" t="str">
         <v>Event</v>
@@ -560,7 +560,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>current</v>
+        <v>previous</v>
       </c>
       <c r="B4" t="str">
         <v>Event</v>
@@ -931,7 +931,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>future</v>
+        <v>current</v>
       </c>
       <c r="B11" t="str">
         <v>Event</v>
@@ -984,7 +984,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>future</v>
       </c>
       <c r="B12" t="str">
         <v>Event</v>

</xml_diff>